<commit_message>
Auto update portfolio 2026-08-14 12:15 UTC
</commit_message>
<xml_diff>
--- a/data/MyPortfolio.xlsx
+++ b/data/MyPortfolio.xlsx
@@ -633,31 +633,31 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>21600</v>
+        <v>21250</v>
       </c>
       <c r="C2" s="9" t="n">
-        <v>31800</v>
+        <v>32000</v>
       </c>
       <c r="D2" s="9" t="n">
-        <v>69000</v>
+        <v>68300</v>
       </c>
       <c r="E2" s="9" t="n">
         <v>36500</v>
       </c>
       <c r="F2" s="10" t="n">
-        <v>142700</v>
+        <v>142900</v>
       </c>
       <c r="G2" s="10" t="n">
-        <v>72600</v>
+        <v>72400</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>20100</v>
+        <v>20000</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>1744.75</v>
+        <v>1729.08</v>
       </c>
       <c r="J2" s="12" t="n">
-        <v>70684000</v>
+        <v>70270000</v>
       </c>
       <c r="K2" s="12" t="n">
         <v>0</v>
@@ -669,25 +669,25 @@
         <v>0</v>
       </c>
       <c r="N2" s="13" t="n">
-        <v>0.0262202735271059</v>
+        <v>0.02020964604082581</v>
       </c>
       <c r="O2" s="13" t="n">
-        <v>-0.0118258072189531</v>
+        <v>-0.02070082633394321</v>
       </c>
       <c r="P2" s="13" t="n">
-        <v>0.5020206674183585</v>
+        <v>0.4932232513650621</v>
       </c>
       <c r="Q2" s="13" t="n">
-        <v>0.1609808977875595</v>
+        <v>0.1541809700573229</v>
       </c>
       <c r="R2" s="13" t="n">
-        <v>-0.4863205760324661</v>
+        <v>-0.4893292241214607</v>
       </c>
       <c r="S2" s="13" t="n">
-        <v>-0.02226966808443787</v>
+        <v>-0.03105088848914772</v>
       </c>
       <c r="T2" s="14">
-        <f>(-0.48632057603246615 - 0.04) / (STDEVP(N2:N153) * SQRT(252))</f>
+        <f>(-0.48932922412146074 - 0.04) / (STDEVP(N2:N153) * SQRT(252))</f>
         <v/>
       </c>
       <c r="U2" s="13" t="n">

</xml_diff>

<commit_message>
Auto update portfolio 2026-08-17 11:27 UTC
</commit_message>
<xml_diff>
--- a/data/MyPortfolio.xlsx
+++ b/data/MyPortfolio.xlsx
@@ -633,31 +633,31 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>21250</v>
+        <v>21200</v>
       </c>
       <c r="C2" s="9" t="n">
-        <v>31700</v>
+        <v>31800</v>
       </c>
       <c r="D2" s="9" t="n">
-        <v>68300</v>
+        <v>68800</v>
       </c>
       <c r="E2" s="9" t="n">
-        <v>36800</v>
+        <v>36200</v>
       </c>
       <c r="F2" s="10" t="n">
-        <v>143000</v>
+        <v>147000</v>
       </c>
       <c r="G2" s="10" t="n">
-        <v>72300</v>
+        <v>73500</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>20000</v>
+        <v>19900</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0</v>
+        <v>1727.46</v>
       </c>
       <c r="J2" s="12" t="n">
-        <v>70720000</v>
+        <v>69948000</v>
       </c>
       <c r="K2" s="12" t="n">
         <v>0</v>
@@ -669,25 +669,25 @@
         <v>0</v>
       </c>
       <c r="N2" s="13" t="n">
-        <v>0.0064038707841184</v>
+        <v>-0.004582325316635833</v>
       </c>
       <c r="O2" s="13" t="n">
-        <v>-1</v>
+        <v>-0.0009369144284820941</v>
       </c>
       <c r="P2" s="13" t="n">
-        <v>0.5027856601186449</v>
+        <v>0.4863808166569428</v>
       </c>
       <c r="Q2" s="13" t="n">
-        <v>0.1615721958510581</v>
+        <v>0.1488921373782501</v>
       </c>
       <c r="R2" s="13" t="n">
-        <v>-0.4860589544595094</v>
+        <v>-0.4916692837462353</v>
       </c>
       <c r="S2" s="13" t="n">
-        <v>-1</v>
+        <v>-0.03195871089218794</v>
       </c>
       <c r="T2" s="14">
-        <f>(-0.4860589544595094 - 0.04) / (STDEVP(N2:N154) * SQRT(252))</f>
+        <f>(-0.4916692837462353 - 0.04) / (STDEVP(N2:N154) * SQRT(252))</f>
         <v/>
       </c>
       <c r="U2" s="13" t="n">

</xml_diff>